<commit_message>
add level windows, composition adjustment and module annotation
</commit_message>
<xml_diff>
--- a/03_Features/c_data/04_hit_robustness.xlsx
+++ b/03_Features/c_data/04_hit_robustness.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t xml:space="preserve">level</t>
   </si>
@@ -36,6 +36,15 @@
     <t xml:space="preserve">p_full</t>
   </si>
   <si>
+    <t xml:space="preserve">confounders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bh_adj_confounders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bh_adj_all_panels</t>
+  </si>
+  <si>
     <t xml:space="preserve">spearman_rho</t>
   </si>
   <si>
@@ -63,18 +72,45 @@
     <t xml:space="preserve">modules</t>
   </si>
   <si>
+    <t xml:space="preserve">T2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_mcsa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME_greenyellow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blood, myofibre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LR_S14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pathways</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_COAGULATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HALLMARK_ESTROGEN_RESPONSE_LATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME_brown</t>
+  </si>
+  <si>
     <t xml:space="preserve">acute</t>
   </si>
   <si>
-    <t xml:space="preserve">d_mcsa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME_greenyellow</t>
+    <t xml:space="preserve">adipose</t>
   </si>
   <si>
     <t xml:space="preserve">HR_S29</t>
   </si>
   <si>
+    <t xml:space="preserve">HALLMARK_XENOBIOTIC_METABOLISM</t>
+  </si>
+  <si>
     <t xml:space="preserve">dropped</t>
   </si>
   <si>
@@ -112,9 +148,6 @@
   </si>
   <si>
     <t xml:space="preserve">LR_S12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LR_S14</t>
   </si>
   <si>
     <t xml:space="preserve">LR_S17</t>
@@ -498,51 +531,349 @@
       <c r="O1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E2" t="n">
         <v>15</v>
       </c>
       <c r="F2" t="n">
+        <v>0.000862581034775395</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.0000718817528979496</v>
+      </c>
+      <c r="H2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.0057836115680374</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.163579011304736</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.589285714285714</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0207943584831616</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.000073425276003363</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.236703797577197</v>
+      </c>
+      <c r="O2" t="n">
+        <v>14</v>
+      </c>
+      <c r="P2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.018312957351157</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.000642559907058141</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.233346692698233</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.564945055177809</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.642857142857143</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.00973994469559528</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.00186991462261574</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.146655395809704</v>
+      </c>
+      <c r="O3" t="n">
+        <v>13</v>
+      </c>
+      <c r="P3" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>23</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.018312957351157</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.000516708515215676</v>
+      </c>
+      <c r="H4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.297289116252775</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.697275471520373</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.767857142857143</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.000829329629136994</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.00455793922150395</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.146655395809704</v>
+      </c>
+      <c r="O4" t="n">
+        <v>13</v>
+      </c>
+      <c r="P4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>23</v>
+      </c>
+      <c r="R4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.0265933783196268</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.00443222971993781</v>
+      </c>
+      <c r="H5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.254962348541038</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.633930054797602</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.764285714285714</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.000907310111684976</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.010955504329416</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.236703797577197</v>
+      </c>
+      <c r="O5" t="n">
+        <v>14</v>
+      </c>
+      <c r="P5" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F6" t="n">
         <v>0.0373000660506198</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G6" t="n">
         <v>0.00310833883755165</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.172570556514772</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.293842050060747</v>
+      </c>
+      <c r="K6" t="n">
         <v>-0.353571428571428</v>
       </c>
-      <c r="I2" t="n">
+      <c r="L6" t="n">
         <v>0.196071678434199</v>
       </c>
-      <c r="J2" t="n">
+      <c r="M6" t="n">
         <v>0.00390077479933552</v>
       </c>
-      <c r="K2" t="n">
+      <c r="N6" t="n">
         <v>0.20558159977165</v>
       </c>
-      <c r="L2" t="n">
+      <c r="O6" t="n">
         <v>6</v>
       </c>
-      <c r="M2" t="n">
+      <c r="P6" t="n">
         <v>15</v>
       </c>
-      <c r="N2" t="s">
-        <v>19</v>
-      </c>
-      <c r="O2" t="b">
+      <c r="Q6" t="s">
+        <v>30</v>
+      </c>
+      <c r="R6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.0413367459281178</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.00217561820674304</v>
+      </c>
+      <c r="H7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.297289116252775</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.697275471520373</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.664285714285714</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.00691068298451917</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.0215978651937539</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.146655395809704</v>
+      </c>
+      <c r="O7" t="n">
+        <v>10</v>
+      </c>
+      <c r="P7" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>23</v>
+      </c>
+      <c r="R7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -571,358 +902,2083 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="F1" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="G1" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="F2" t="n">
-        <v>0.054979544790258</v>
+        <v>0.00118163529920899</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.0781075050880027</v>
+        <v>0.073124299300869</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0080556933269047</v>
+        <v>0.000073425276003363</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0947387520122267</v>
+        <v>0.0872822004612168</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0503005515198805</v>
+        <v>0.00147484610885631</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0795078627552937</v>
+        <v>0.0727577802279967</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0651213066913984</v>
+        <v>0.00056699920504983</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.079545875114398</v>
+        <v>0.0790348966518401</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="F6" t="n">
-        <v>0.00390077479933552</v>
+        <v>0.000339269112267988</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.08834557932743</v>
+        <v>0.0786728723329441</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="F7" t="n">
-        <v>0.054250679610068</v>
+        <v>0.00168729460596945</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0769331196801686</v>
+        <v>0.070109200198181</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F8" t="n">
-        <v>0.20558159977165</v>
+        <v>0.0122995181487444</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.0654473842144298</v>
+        <v>0.0636658632039701</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0307667424368695</v>
+        <v>0.000996665532841444</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0818500365405104</v>
+        <v>0.0704149903033648</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="F10" t="n">
-        <v>0.127055749489571</v>
+        <v>0.00589897721660364</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0868945680298544</v>
+        <v>0.0801058050779618</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0525059524609568</v>
+        <v>0.00410878433875772</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.0803392131091439</v>
+        <v>0.0711720483689237</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F12" t="n">
-        <v>0.10102433804239</v>
+        <v>0.00188248579220867</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.074790060996202</v>
+        <v>0.0728196418569135</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F13" t="n">
-        <v>0.194280725253742</v>
+        <v>0.236703797577197</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0573831168990567</v>
+        <v>0.0504925265280276</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D14" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0218128597619647</v>
+        <v>0.0185501231274451</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0849230746068681</v>
+        <v>0.075672600452179</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E15" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0477084409451729</v>
+        <v>0.00108568102787966</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.0803503121684322</v>
+        <v>0.0743525658254965</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C16" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D16" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E16" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.000863553705804061</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.0754896132847661</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" t="s">
+        <v>35</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.0180593118327047</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.00960496156320465</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" t="s">
         <v>36</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F18" t="n">
+        <v>0.0203896096751573</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0108208330842879</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.0292187142738882</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.009688648955494</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" t="s">
+        <v>38</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.0335558909838178</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.00971556845516111</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" t="s">
+        <v>39</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.00186991462261574</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.0106949775858962</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" t="s">
+        <v>40</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.0249032258584645</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.00960438171784701</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.03724115772407</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.00894112567696815</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" t="s">
+        <v>41</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.0231827687759881</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.0101635216761814</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" t="s">
+        <v>42</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.0929292442864682</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.0100613927188519</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" t="s">
+        <v>43</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.0271186068072054</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.00984026757509056</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" t="s">
+        <v>44</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.0386141805267378</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.00959624044769593</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>24</v>
+      </c>
+      <c r="B28" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" t="s">
+        <v>20</v>
+      </c>
+      <c r="D28" t="s">
+        <v>25</v>
+      </c>
+      <c r="E28" t="s">
+        <v>23</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.146655395809704</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.00726663829573475</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" t="s">
+        <v>25</v>
+      </c>
+      <c r="E29" t="s">
+        <v>45</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.0215978651937539</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.0102705738881989</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" t="s">
+        <v>25</v>
+      </c>
+      <c r="E30" t="s">
+        <v>46</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.0272816226359498</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.00980054625176529</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>24</v>
+      </c>
+      <c r="B31" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" t="s">
+        <v>25</v>
+      </c>
+      <c r="E31" t="s">
+        <v>47</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.0298262535942641</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.00975987150161447</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>24</v>
+      </c>
+      <c r="B32" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32" t="s">
+        <v>26</v>
+      </c>
+      <c r="E32" t="s">
+        <v>35</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.0180593118327047</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.00575419140373489</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>24</v>
+      </c>
+      <c r="B33" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" t="s">
+        <v>26</v>
+      </c>
+      <c r="E33" t="s">
+        <v>36</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.0305362210249045</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.005655378271936</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>24</v>
+      </c>
+      <c r="B34" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" t="s">
+        <v>26</v>
+      </c>
+      <c r="E34" t="s">
+        <v>37</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.0292187142738882</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.00557769520349468</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>24</v>
+      </c>
+      <c r="B35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" t="s">
+        <v>26</v>
+      </c>
+      <c r="E35" t="s">
+        <v>38</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.0281065062313901</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.00602686155525983</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>24</v>
+      </c>
+      <c r="B36" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" t="s">
+        <v>26</v>
+      </c>
+      <c r="E36" t="s">
+        <v>39</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.00455793922150395</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.00605825737202629</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B37" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" t="s">
+        <v>26</v>
+      </c>
+      <c r="E37" t="s">
+        <v>40</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.0249032258584645</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.0056406425988425</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>24</v>
+      </c>
+      <c r="B38" t="s">
+        <v>19</v>
+      </c>
+      <c r="C38" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" t="s">
+        <v>26</v>
+      </c>
+      <c r="E38" t="s">
+        <v>30</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.0262355883900738</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.0058210047311981</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>24</v>
+      </c>
+      <c r="B39" t="s">
+        <v>19</v>
+      </c>
+      <c r="C39" t="s">
+        <v>20</v>
+      </c>
+      <c r="D39" t="s">
+        <v>26</v>
+      </c>
+      <c r="E39" t="s">
+        <v>41</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.0250651087844653</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.00560464641328965</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>24</v>
+      </c>
+      <c r="B40" t="s">
+        <v>19</v>
+      </c>
+      <c r="C40" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" t="s">
+        <v>26</v>
+      </c>
+      <c r="E40" t="s">
+        <v>42</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.0929292442864682</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.00583494788180694</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>24</v>
+      </c>
+      <c r="B41" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" t="s">
+        <v>20</v>
+      </c>
+      <c r="D41" t="s">
+        <v>26</v>
+      </c>
+      <c r="E41" t="s">
+        <v>43</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.0232068562153472</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.00597569351701983</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>24</v>
+      </c>
+      <c r="B42" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" t="s">
+        <v>20</v>
+      </c>
+      <c r="D42" t="s">
+        <v>26</v>
+      </c>
+      <c r="E42" t="s">
+        <v>44</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.0386141805267378</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.00553266543587009</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>24</v>
+      </c>
+      <c r="B43" t="s">
+        <v>19</v>
+      </c>
+      <c r="C43" t="s">
+        <v>20</v>
+      </c>
+      <c r="D43" t="s">
+        <v>26</v>
+      </c>
+      <c r="E43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.146655395809704</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.0048769256346904</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>24</v>
+      </c>
+      <c r="B44" t="s">
+        <v>19</v>
+      </c>
+      <c r="C44" t="s">
+        <v>20</v>
+      </c>
+      <c r="D44" t="s">
+        <v>26</v>
+      </c>
+      <c r="E44" t="s">
+        <v>45</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.0244675491908857</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.00542232799765981</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>24</v>
+      </c>
+      <c r="B45" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" t="s">
+        <v>20</v>
+      </c>
+      <c r="D45" t="s">
+        <v>26</v>
+      </c>
+      <c r="E45" t="s">
+        <v>46</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.0272816226359498</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.00579537339481097</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>24</v>
+      </c>
+      <c r="B46" t="s">
+        <v>19</v>
+      </c>
+      <c r="C46" t="s">
+        <v>20</v>
+      </c>
+      <c r="D46" t="s">
+        <v>26</v>
+      </c>
+      <c r="E46" t="s">
+        <v>47</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.0298262535942641</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.005530380125017</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>18</v>
+      </c>
+      <c r="B47" t="s">
+        <v>19</v>
+      </c>
+      <c r="C47" t="s">
+        <v>20</v>
+      </c>
+      <c r="D47" t="s">
+        <v>27</v>
+      </c>
+      <c r="E47" t="s">
+        <v>35</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.0324297204114665</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.051555175206641</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>18</v>
+      </c>
+      <c r="B48" t="s">
+        <v>19</v>
+      </c>
+      <c r="C48" t="s">
+        <v>20</v>
+      </c>
+      <c r="D48" t="s">
+        <v>27</v>
+      </c>
+      <c r="E48" t="s">
+        <v>36</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.010955504329416</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.0590302927311564</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>18</v>
+      </c>
+      <c r="B49" t="s">
+        <v>19</v>
+      </c>
+      <c r="C49" t="s">
+        <v>20</v>
+      </c>
+      <c r="D49" t="s">
+        <v>27</v>
+      </c>
+      <c r="E49" t="s">
+        <v>37</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.0333633163196286</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.0518803022847024</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>18</v>
+      </c>
+      <c r="B50" t="s">
+        <v>19</v>
+      </c>
+      <c r="C50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D50" t="s">
+        <v>27</v>
+      </c>
+      <c r="E50" t="s">
+        <v>38</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.0374529128045459</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.0522773391659244</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>18</v>
+      </c>
+      <c r="B51" t="s">
+        <v>19</v>
+      </c>
+      <c r="C51" t="s">
+        <v>20</v>
+      </c>
+      <c r="D51" t="s">
+        <v>27</v>
+      </c>
+      <c r="E51" t="s">
+        <v>39</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.0185420938998591</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.0547363544279826</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>18</v>
+      </c>
+      <c r="B52" t="s">
+        <v>19</v>
+      </c>
+      <c r="C52" t="s">
+        <v>20</v>
+      </c>
+      <c r="D52" t="s">
+        <v>27</v>
+      </c>
+      <c r="E52" t="s">
+        <v>40</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.0284447297497447</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.0514131422604534</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>18</v>
+      </c>
+      <c r="B53" t="s">
+        <v>19</v>
+      </c>
+      <c r="C53" t="s">
+        <v>20</v>
+      </c>
+      <c r="D53" t="s">
+        <v>27</v>
+      </c>
+      <c r="E53" t="s">
+        <v>30</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.036248812154879</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.052930301314676</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54" t="s">
+        <v>19</v>
+      </c>
+      <c r="C54" t="s">
+        <v>20</v>
+      </c>
+      <c r="D54" t="s">
+        <v>27</v>
+      </c>
+      <c r="E54" t="s">
+        <v>41</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.0189706078846877</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.0521832430421757</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>18</v>
+      </c>
+      <c r="B55" t="s">
+        <v>19</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55" t="s">
+        <v>27</v>
+      </c>
+      <c r="E55" t="s">
+        <v>42</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.0352798108372291</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.0628004454117927</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>18</v>
+      </c>
+      <c r="B56" t="s">
+        <v>19</v>
+      </c>
+      <c r="C56" t="s">
+        <v>20</v>
+      </c>
+      <c r="D56" t="s">
+        <v>27</v>
+      </c>
+      <c r="E56" t="s">
+        <v>43</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.0241925589050649</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.0522198016369385</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>18</v>
+      </c>
+      <c r="B57" t="s">
+        <v>19</v>
+      </c>
+      <c r="C57" t="s">
+        <v>20</v>
+      </c>
+      <c r="D57" t="s">
+        <v>27</v>
+      </c>
+      <c r="E57" t="s">
+        <v>44</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.045421229947806</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.0508049476725222</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>18</v>
+      </c>
+      <c r="B58" t="s">
+        <v>19</v>
+      </c>
+      <c r="C58" t="s">
+        <v>20</v>
+      </c>
+      <c r="D58" t="s">
+        <v>27</v>
+      </c>
+      <c r="E58" t="s">
+        <v>23</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.236703797577197</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0.0299888701728618</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>18</v>
+      </c>
+      <c r="B59" t="s">
+        <v>19</v>
+      </c>
+      <c r="C59" t="s">
+        <v>20</v>
+      </c>
+      <c r="D59" t="s">
+        <v>27</v>
+      </c>
+      <c r="E59" t="s">
+        <v>45</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.0275573330981754</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.0487493764814065</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>18</v>
+      </c>
+      <c r="B60" t="s">
+        <v>19</v>
+      </c>
+      <c r="C60" t="s">
+        <v>20</v>
+      </c>
+      <c r="D60" t="s">
+        <v>27</v>
+      </c>
+      <c r="E60" t="s">
+        <v>46</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.0297352136625235</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0.0526719816945665</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>18</v>
+      </c>
+      <c r="B61" t="s">
+        <v>19</v>
+      </c>
+      <c r="C61" t="s">
+        <v>20</v>
+      </c>
+      <c r="D61" t="s">
+        <v>27</v>
+      </c>
+      <c r="E61" t="s">
+        <v>47</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.0297918549492885</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.0526858422997235</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>18</v>
+      </c>
+      <c r="B62" t="s">
+        <v>28</v>
+      </c>
+      <c r="C62" t="s">
+        <v>20</v>
+      </c>
+      <c r="D62" t="s">
+        <v>21</v>
+      </c>
+      <c r="E62" t="s">
+        <v>35</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.054979544790258</v>
+      </c>
+      <c r="G62" t="n">
+        <v>-0.0781075050880027</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>18</v>
+      </c>
+      <c r="B63" t="s">
+        <v>28</v>
+      </c>
+      <c r="C63" t="s">
+        <v>20</v>
+      </c>
+      <c r="D63" t="s">
+        <v>21</v>
+      </c>
+      <c r="E63" t="s">
+        <v>36</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.0080556933269047</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-0.0947387520122267</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>18</v>
+      </c>
+      <c r="B64" t="s">
+        <v>28</v>
+      </c>
+      <c r="C64" t="s">
+        <v>20</v>
+      </c>
+      <c r="D64" t="s">
+        <v>21</v>
+      </c>
+      <c r="E64" t="s">
+        <v>37</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.0503005515198805</v>
+      </c>
+      <c r="G64" t="n">
+        <v>-0.0795078627552937</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>18</v>
+      </c>
+      <c r="B65" t="s">
+        <v>28</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65" t="s">
+        <v>21</v>
+      </c>
+      <c r="E65" t="s">
+        <v>38</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.0651213066913984</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-0.079545875114398</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>18</v>
+      </c>
+      <c r="B66" t="s">
+        <v>28</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66" t="s">
+        <v>21</v>
+      </c>
+      <c r="E66" t="s">
+        <v>39</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.00390077479933552</v>
+      </c>
+      <c r="G66" t="n">
+        <v>-0.08834557932743</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>18</v>
+      </c>
+      <c r="B67" t="s">
+        <v>28</v>
+      </c>
+      <c r="C67" t="s">
+        <v>20</v>
+      </c>
+      <c r="D67" t="s">
+        <v>21</v>
+      </c>
+      <c r="E67" t="s">
+        <v>40</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.054250679610068</v>
+      </c>
+      <c r="G67" t="n">
+        <v>-0.0769331196801686</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>18</v>
+      </c>
+      <c r="B68" t="s">
+        <v>28</v>
+      </c>
+      <c r="C68" t="s">
+        <v>20</v>
+      </c>
+      <c r="D68" t="s">
+        <v>21</v>
+      </c>
+      <c r="E68" t="s">
+        <v>30</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.20558159977165</v>
+      </c>
+      <c r="G68" t="n">
+        <v>-0.0654473842144298</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>18</v>
+      </c>
+      <c r="B69" t="s">
+        <v>28</v>
+      </c>
+      <c r="C69" t="s">
+        <v>20</v>
+      </c>
+      <c r="D69" t="s">
+        <v>21</v>
+      </c>
+      <c r="E69" t="s">
+        <v>41</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.0307667424368695</v>
+      </c>
+      <c r="G69" t="n">
+        <v>-0.0818500365405104</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>18</v>
+      </c>
+      <c r="B70" t="s">
+        <v>28</v>
+      </c>
+      <c r="C70" t="s">
+        <v>20</v>
+      </c>
+      <c r="D70" t="s">
+        <v>21</v>
+      </c>
+      <c r="E70" t="s">
+        <v>42</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.127055749489571</v>
+      </c>
+      <c r="G70" t="n">
+        <v>-0.0868945680298544</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>18</v>
+      </c>
+      <c r="B71" t="s">
+        <v>28</v>
+      </c>
+      <c r="C71" t="s">
+        <v>20</v>
+      </c>
+      <c r="D71" t="s">
+        <v>21</v>
+      </c>
+      <c r="E71" t="s">
+        <v>43</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.0525059524609568</v>
+      </c>
+      <c r="G71" t="n">
+        <v>-0.0803392131091439</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>18</v>
+      </c>
+      <c r="B72" t="s">
+        <v>28</v>
+      </c>
+      <c r="C72" t="s">
+        <v>20</v>
+      </c>
+      <c r="D72" t="s">
+        <v>21</v>
+      </c>
+      <c r="E72" t="s">
+        <v>44</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.10102433804239</v>
+      </c>
+      <c r="G72" t="n">
+        <v>-0.074790060996202</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>18</v>
+      </c>
+      <c r="B73" t="s">
+        <v>28</v>
+      </c>
+      <c r="C73" t="s">
+        <v>20</v>
+      </c>
+      <c r="D73" t="s">
+        <v>21</v>
+      </c>
+      <c r="E73" t="s">
+        <v>23</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0.194280725253742</v>
+      </c>
+      <c r="G73" t="n">
+        <v>-0.0573831168990567</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
+        <v>18</v>
+      </c>
+      <c r="B74" t="s">
+        <v>28</v>
+      </c>
+      <c r="C74" t="s">
+        <v>20</v>
+      </c>
+      <c r="D74" t="s">
+        <v>21</v>
+      </c>
+      <c r="E74" t="s">
+        <v>45</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0.0218128597619647</v>
+      </c>
+      <c r="G74" t="n">
+        <v>-0.0849230746068681</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s">
+        <v>18</v>
+      </c>
+      <c r="B75" t="s">
+        <v>28</v>
+      </c>
+      <c r="C75" t="s">
+        <v>20</v>
+      </c>
+      <c r="D75" t="s">
+        <v>21</v>
+      </c>
+      <c r="E75" t="s">
+        <v>46</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0.0477084409451729</v>
+      </c>
+      <c r="G75" t="n">
+        <v>-0.0803503121684322</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s">
+        <v>18</v>
+      </c>
+      <c r="B76" t="s">
+        <v>28</v>
+      </c>
+      <c r="C76" t="s">
+        <v>20</v>
+      </c>
+      <c r="D76" t="s">
+        <v>21</v>
+      </c>
+      <c r="E76" t="s">
+        <v>47</v>
+      </c>
+      <c r="F76" t="n">
         <v>0.0313306865487702</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G76" t="n">
         <v>-0.0821250609064925</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s">
+        <v>24</v>
+      </c>
+      <c r="B77" t="s">
+        <v>19</v>
+      </c>
+      <c r="C77" t="s">
+        <v>20</v>
+      </c>
+      <c r="D77" t="s">
+        <v>31</v>
+      </c>
+      <c r="E77" t="s">
+        <v>35</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.0496120322211278</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0.00467631014096833</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s">
+        <v>24</v>
+      </c>
+      <c r="B78" t="s">
+        <v>19</v>
+      </c>
+      <c r="C78" t="s">
+        <v>20</v>
+      </c>
+      <c r="D78" t="s">
+        <v>31</v>
+      </c>
+      <c r="E78" t="s">
+        <v>36</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0.0477173337817574</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0.00482900159249192</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>24</v>
+      </c>
+      <c r="B79" t="s">
+        <v>19</v>
+      </c>
+      <c r="C79" t="s">
+        <v>20</v>
+      </c>
+      <c r="D79" t="s">
+        <v>31</v>
+      </c>
+      <c r="E79" t="s">
+        <v>37</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0.0488316283083433</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0.004548916608998</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>24</v>
+      </c>
+      <c r="B80" t="s">
+        <v>19</v>
+      </c>
+      <c r="C80" t="s">
+        <v>20</v>
+      </c>
+      <c r="D80" t="s">
+        <v>31</v>
+      </c>
+      <c r="E80" t="s">
+        <v>38</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0.0938682706358487</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0.00447284766295817</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s">
+        <v>24</v>
+      </c>
+      <c r="B81" t="s">
+        <v>19</v>
+      </c>
+      <c r="C81" t="s">
+        <v>20</v>
+      </c>
+      <c r="D81" t="s">
+        <v>31</v>
+      </c>
+      <c r="E81" t="s">
+        <v>39</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0.0497500231913178</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0.00450254948858384</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s">
+        <v>24</v>
+      </c>
+      <c r="B82" t="s">
+        <v>19</v>
+      </c>
+      <c r="C82" t="s">
+        <v>20</v>
+      </c>
+      <c r="D82" t="s">
+        <v>31</v>
+      </c>
+      <c r="E82" t="s">
+        <v>40</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0.0430662476375439</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0.0046226304413178</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s">
+        <v>24</v>
+      </c>
+      <c r="B83" t="s">
+        <v>19</v>
+      </c>
+      <c r="C83" t="s">
+        <v>20</v>
+      </c>
+      <c r="D83" t="s">
+        <v>31</v>
+      </c>
+      <c r="E83" t="s">
+        <v>30</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0.0262355883900738</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0.00524173739453877</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
+        <v>24</v>
+      </c>
+      <c r="B84" t="s">
+        <v>19</v>
+      </c>
+      <c r="C84" t="s">
+        <v>20</v>
+      </c>
+      <c r="D84" t="s">
+        <v>31</v>
+      </c>
+      <c r="E84" t="s">
+        <v>41</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0.0477441876421588</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0.00423432632961194</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s">
+        <v>24</v>
+      </c>
+      <c r="B85" t="s">
+        <v>19</v>
+      </c>
+      <c r="C85" t="s">
+        <v>20</v>
+      </c>
+      <c r="D85" t="s">
+        <v>31</v>
+      </c>
+      <c r="E85" t="s">
+        <v>42</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0.122010651297781</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0.00403432365758341</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s">
+        <v>24</v>
+      </c>
+      <c r="B86" t="s">
+        <v>19</v>
+      </c>
+      <c r="C86" t="s">
+        <v>20</v>
+      </c>
+      <c r="D86" t="s">
+        <v>31</v>
+      </c>
+      <c r="E86" t="s">
+        <v>43</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0.0389745706244434</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0.00481960192901435</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="s">
+        <v>24</v>
+      </c>
+      <c r="B87" t="s">
+        <v>19</v>
+      </c>
+      <c r="C87" t="s">
+        <v>20</v>
+      </c>
+      <c r="D87" t="s">
+        <v>31</v>
+      </c>
+      <c r="E87" t="s">
+        <v>44</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0.0928626427354628</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0.00443442771932531</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="s">
+        <v>24</v>
+      </c>
+      <c r="B88" t="s">
+        <v>19</v>
+      </c>
+      <c r="C88" t="s">
+        <v>20</v>
+      </c>
+      <c r="D88" t="s">
+        <v>31</v>
+      </c>
+      <c r="E88" t="s">
+        <v>23</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0.146655395809704</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0.00437001415395459</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="s">
+        <v>24</v>
+      </c>
+      <c r="B89" t="s">
+        <v>19</v>
+      </c>
+      <c r="C89" t="s">
+        <v>20</v>
+      </c>
+      <c r="D89" t="s">
+        <v>31</v>
+      </c>
+      <c r="E89" t="s">
+        <v>45</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0.0215978651937539</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0.00520739611656507</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="s">
+        <v>24</v>
+      </c>
+      <c r="B90" t="s">
+        <v>19</v>
+      </c>
+      <c r="C90" t="s">
+        <v>20</v>
+      </c>
+      <c r="D90" t="s">
+        <v>31</v>
+      </c>
+      <c r="E90" t="s">
+        <v>46</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0.0364032423872812</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0.00478027194678659</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s">
+        <v>24</v>
+      </c>
+      <c r="B91" t="s">
+        <v>19</v>
+      </c>
+      <c r="C91" t="s">
+        <v>20</v>
+      </c>
+      <c r="D91" t="s">
+        <v>31</v>
+      </c>
+      <c r="E91" t="s">
+        <v>47</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0.0592923158689442</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0.00464346619027562</v>
       </c>
     </row>
   </sheetData>

</xml_diff>